<commit_message>
Add lead & personalized demo for McMullinPlumbingss
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="99">
   <si>
     <t>Niche</t>
   </si>
@@ -281,6 +281,36 @@
   </si>
   <si>
     <t>Full-service residential &amp; commercial plumbing contractor in Lakeland/Memphis TN. Owned by Master Plumber Bill McMullin ("Mr. Bill"). Specializes in water heater installation &amp; repair (Mr. Bill's Water Heater Deals), leak detection, drain cleaning, tankless upgrades, emergency repairs.</t>
+  </si>
+  <si>
+    <t>South Charleston, West Virginia</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/MullenPlumbing</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/mullen_plumbing_hvac</t>
+  </si>
+  <si>
+    <t>https://mullenplumbing.com</t>
+  </si>
+  <si>
+    <t>Mullen Plumbing, Heating &amp; Cooling</t>
+  </si>
+  <si>
+    <t>Tom Orcutt</t>
+  </si>
+  <si>
+    <t>(304) 744-3221</t>
+  </si>
+  <si>
+    <t>Tom.Orcutt@mullenplumbing.com</t>
+  </si>
+  <si>
+    <t>https://master-five-theta.vercel.app/coldemail/MullenPlumbingHeatingCooling/index.html</t>
+  </si>
+  <si>
+    <t>Full-service 24/7 residential &amp; commercial plumbing &amp; HVAC contractor in South Charleston/Charleston WV founded in 1950 (75+ yrs exp). Led by President Tom Orcutt. Services include 24/7 emergency plumbing, water heaters, sewer/drain cleaning, heating &amp; AC repair/installation.</t>
   </si>
 </sst>
 </file>
@@ -642,7 +672,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -1046,6 +1076,74 @@
         <v>88</v>
       </c>
     </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" t="s">
+        <v>94</v>
+      </c>
+      <c r="I8" t="s">
+        <v>95</v>
+      </c>
+      <c r="J8" t="s">
+        <v>96</v>
+      </c>
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" t="s">
+        <v>97</v>
+      </c>
+      <c r="N8" t="s">
+        <v>86</v>
+      </c>
+      <c r="O8" t="s">
+        <v>34</v>
+      </c>
+      <c r="P8" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>87</v>
+      </c>
+      <c r="R8" t="s">
+        <v>87</v>
+      </c>
+      <c r="S8" t="s">
+        <v>87</v>
+      </c>
+      <c r="T8" t="s">
+        <v>35</v>
+      </c>
+      <c r="U8" t="s">
+        <v>87</v>
+      </c>
+      <c r="V8" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lead & personalized demo for McMullinPlumbingssjjh
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="110">
   <si>
     <t>Niche</t>
   </si>
@@ -311,6 +311,39 @@
   </si>
   <si>
     <t>Full-service 24/7 residential &amp; commercial plumbing &amp; HVAC contractor in South Charleston/Charleston WV founded in 1950 (75+ yrs exp). Led by President Tom Orcutt. Services include 24/7 emergency plumbing, water heaters, sewer/drain cleaning, heating &amp; AC repair/installation.</t>
+  </si>
+  <si>
+    <t>Gibson, Tennessee</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/McMillionPlumbing</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/mcmillionplumbing</t>
+  </si>
+  <si>
+    <t>https://www.mcmillionplumbing.com</t>
+  </si>
+  <si>
+    <t>Mcmillion Plumbing</t>
+  </si>
+  <si>
+    <t>Bret McMillion</t>
+  </si>
+  <si>
+    <t>(731) 234-0775</t>
+  </si>
+  <si>
+    <t>beneshia@mcmillionplumbing.com</t>
+  </si>
+  <si>
+    <t>bret@mcmillionconstruction.com</t>
+  </si>
+  <si>
+    <t>https://master-five-theta.vercel.app/coldemail/McmillionPlumbing/index.html</t>
+  </si>
+  <si>
+    <t>Full-service residential &amp; commercial plumbing contractor in Gibson/Humboldt TN founded in 2014 (10+ yrs exp, A+ BBB Accredited). Owned by Bret McMillion, managed by Beneshia McMillion. Services include emergency plumbing repairs, water heaters, sewer/drain cleaning, leak detection, piping.</t>
   </si>
 </sst>
 </file>
@@ -672,7 +705,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -1144,6 +1177,74 @@
         <v>98</v>
       </c>
     </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" t="s">
+        <v>106</v>
+      </c>
+      <c r="K9" t="s">
+        <v>107</v>
+      </c>
+      <c r="L9" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" t="s">
+        <v>108</v>
+      </c>
+      <c r="N9" t="s">
+        <v>86</v>
+      </c>
+      <c r="O9" t="s">
+        <v>34</v>
+      </c>
+      <c r="P9" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>87</v>
+      </c>
+      <c r="R9" t="s">
+        <v>87</v>
+      </c>
+      <c r="S9" t="s">
+        <v>87</v>
+      </c>
+      <c r="T9" t="s">
+        <v>35</v>
+      </c>
+      <c r="U9" t="s">
+        <v>87</v>
+      </c>
+      <c r="V9" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lead & personalized demo for McMullinPlumbingssjjhssss
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="122">
   <si>
     <t>Niche</t>
   </si>
@@ -344,6 +344,42 @@
   </si>
   <si>
     <t>Full-service residential &amp; commercial plumbing contractor in Gibson/Humboldt TN founded in 2014 (10+ yrs exp, A+ BBB Accredited). Owned by Bret McMillion, managed by Beneshia McMillion. Services include emergency plumbing repairs, water heaters, sewer/drain cleaning, leak detection, piping.</t>
+  </si>
+  <si>
+    <t>Covington, Kentucky</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/people/A-Plumbing/100063901768407/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/maximumplumbingky/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/kadin-sarieh</t>
+  </si>
+  <si>
+    <t>https://callaplusnow.com</t>
+  </si>
+  <si>
+    <t>A+ Plumbing</t>
+  </si>
+  <si>
+    <t>Gary Geiman</t>
+  </si>
+  <si>
+    <t>(859) 212-9512</t>
+  </si>
+  <si>
+    <t>info@callaplusnow.com</t>
+  </si>
+  <si>
+    <t>callaplusnow@outlook.com</t>
+  </si>
+  <si>
+    <t>https://master-five-theta.vercel.app/coldemail/APlusPlumbing/index.html</t>
+  </si>
+  <si>
+    <t>Full-service 24/7 emergency residential &amp; commercial plumbing contractor in Covington/Latonia KY &amp; Greater Cincinnati. Owned &amp; operated by Master Plumber Gary Geiman (KY Lic #M8032, A+ BBB Accredited, 1,074+ Google reviews at 4.9 stars). Services include 24/7 emergency plumbing, water heaters, sewer/drain cleaning, leak detection, water restoration.</t>
   </si>
 </sst>
 </file>
@@ -705,7 +741,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -1245,6 +1281,74 @@
         <v>109</v>
       </c>
     </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>113</v>
+      </c>
+      <c r="F10" t="s">
+        <v>114</v>
+      </c>
+      <c r="G10" t="s">
+        <v>115</v>
+      </c>
+      <c r="H10" t="s">
+        <v>116</v>
+      </c>
+      <c r="I10" t="s">
+        <v>117</v>
+      </c>
+      <c r="J10" t="s">
+        <v>118</v>
+      </c>
+      <c r="K10" t="s">
+        <v>119</v>
+      </c>
+      <c r="L10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" t="s">
+        <v>120</v>
+      </c>
+      <c r="N10" t="s">
+        <v>86</v>
+      </c>
+      <c r="O10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P10" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>87</v>
+      </c>
+      <c r="R10" t="s">
+        <v>87</v>
+      </c>
+      <c r="S10" t="s">
+        <v>87</v>
+      </c>
+      <c r="T10" t="s">
+        <v>35</v>
+      </c>
+      <c r="U10" t="s">
+        <v>87</v>
+      </c>
+      <c r="V10" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lead & personalized demo for McMullinPlumbingssjjhsssssdsds
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="132">
   <si>
     <t>Niche</t>
   </si>
@@ -349,13 +349,10 @@
     <t>Covington, Kentucky</t>
   </si>
   <si>
-    <t>https://www.facebook.com/people/A-Plumbing/100063901768407/</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/maximumplumbingky/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/kadin-sarieh</t>
+    <t>https://www.linkedin.com/in/kadin-sarieh-979146237/</t>
   </si>
   <si>
     <t>https://callaplusnow.com</t>
@@ -380,6 +377,39 @@
   </si>
   <si>
     <t>Full-service 24/7 emergency residential &amp; commercial plumbing contractor in Covington/Latonia KY &amp; Greater Cincinnati. Owned &amp; operated by Master Plumber Gary Geiman (KY Lic #M8032, A+ BBB Accredited, 1,074+ Google reviews at 4.9 stars). Services include 24/7 emergency plumbing, water heaters, sewer/drain cleaning, leak detection, water restoration.</t>
+  </si>
+  <si>
+    <t>San Antonio, Texas</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/sewertvhydrojettingplumbingsanantonio</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/sewertvplumber/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/company/sewertv-plumbing-san-antonio/</t>
+  </si>
+  <si>
+    <t>https://sewertvplumbing.com</t>
+  </si>
+  <si>
+    <t>SewerTV Hydro Jetting and Plumbing</t>
+  </si>
+  <si>
+    <t>Dave</t>
+  </si>
+  <si>
+    <t>(210) 500-9840</t>
+  </si>
+  <si>
+    <t>dave@sewertvplumbing.com</t>
+  </si>
+  <si>
+    <t>https://master-five-theta.vercel.app/coldemail/SewerTVHydroJettingandPlumbing/index.html</t>
+  </si>
+  <si>
+    <t>Full-service 24/7 emergency residential &amp; commercial plumbing contractor in San Antonio TX founded in 2002 (20+ yrs exp, Texas Master Plumber Lic #44506, 140+ Google reviews at 4.9 stars). Owned &amp; operated by Dave. Services include 24/7 emergency plumbing, high-pressure hydro jetting, sewer camera inspection, trenchless pipe lining, water line repair.</t>
   </si>
 </sst>
 </file>
@@ -741,7 +771,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -1289,37 +1319,37 @@
         <v>110</v>
       </c>
       <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
         <v>111</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>112</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>113</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>114</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>115</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>116</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>117</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>118</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" t="s">
         <v>119</v>
-      </c>
-      <c r="L10" t="s">
-        <v>25</v>
-      </c>
-      <c r="M10" t="s">
-        <v>120</v>
       </c>
       <c r="N10" t="s">
         <v>86</v>
@@ -1346,7 +1376,75 @@
         <v>87</v>
       </c>
       <c r="V10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
         <v>121</v>
+      </c>
+      <c r="C11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" t="s">
+        <v>126</v>
+      </c>
+      <c r="H11" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" t="s">
+        <v>128</v>
+      </c>
+      <c r="J11" t="s">
+        <v>129</v>
+      </c>
+      <c r="K11" t="s">
+        <v>25</v>
+      </c>
+      <c r="L11" t="s">
+        <v>25</v>
+      </c>
+      <c r="M11" t="s">
+        <v>130</v>
+      </c>
+      <c r="N11" t="s">
+        <v>86</v>
+      </c>
+      <c r="O11" t="s">
+        <v>34</v>
+      </c>
+      <c r="P11" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>87</v>
+      </c>
+      <c r="R11" t="s">
+        <v>87</v>
+      </c>
+      <c r="S11" t="s">
+        <v>87</v>
+      </c>
+      <c r="T11" t="s">
+        <v>35</v>
+      </c>
+      <c r="U11" t="s">
+        <v>87</v>
+      </c>
+      <c r="V11" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add lead & personalized demo for McMullinPlumbingssjjhsssssdsdsvbhvhvbh
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="143">
   <si>
     <t>Niche</t>
   </si>
@@ -410,6 +410,39 @@
   </si>
   <si>
     <t>Full-service 24/7 emergency residential &amp; commercial plumbing contractor in San Antonio TX founded in 2002 (20+ yrs exp, Texas Master Plumber Lic #44506, 140+ Google reviews at 4.9 stars). Owned &amp; operated by Dave. Services include 24/7 emergency plumbing, high-pressure hydro jetting, sewer camera inspection, trenchless pipe lining, water line repair.</t>
+  </si>
+  <si>
+    <t>Springfield, Missouri</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/reedsplumbingmo/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/reedsplumbingmo/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/company/reeds-plumbing</t>
+  </si>
+  <si>
+    <t>https://www.reedsplumbing.com</t>
+  </si>
+  <si>
+    <t>Reed’s Plumbing, Excavating, Septic, Heating &amp; Air</t>
+  </si>
+  <si>
+    <t>Titus Williams</t>
+  </si>
+  <si>
+    <t>(417) 831-6122</t>
+  </si>
+  <si>
+    <t>office@reedsplumbing.com</t>
+  </si>
+  <si>
+    <t>https://master-five-theta.vercel.app/coldemail/ReedsPlumbingExcavatingSepticHeatingAir/index.html</t>
+  </si>
+  <si>
+    <t>Full-service 24/7 emergency residential &amp; commercial plumbing, septic, excavation &amp; HVAC contractor in Springfield MO operating since 1972 (50+ yrs exp, A+ BBB Accredited since 1998, 925+ Google reviews at 4.8 stars). Owned by Titus Williams, managed by GM Mike Lile. Services include 24/7 emergency plumbing, water heaters, septic pumping, excavation, heating &amp; AC repair/installation.</t>
   </si>
 </sst>
 </file>
@@ -771,7 +804,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -1447,6 +1480,74 @@
         <v>131</v>
       </c>
     </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F12" t="s">
+        <v>136</v>
+      </c>
+      <c r="G12" t="s">
+        <v>137</v>
+      </c>
+      <c r="H12" t="s">
+        <v>138</v>
+      </c>
+      <c r="I12" t="s">
+        <v>139</v>
+      </c>
+      <c r="J12" t="s">
+        <v>140</v>
+      </c>
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" t="s">
+        <v>141</v>
+      </c>
+      <c r="N12" t="s">
+        <v>86</v>
+      </c>
+      <c r="O12" t="s">
+        <v>34</v>
+      </c>
+      <c r="P12" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>87</v>
+      </c>
+      <c r="R12" t="s">
+        <v>87</v>
+      </c>
+      <c r="S12" t="s">
+        <v>87</v>
+      </c>
+      <c r="T12" t="s">
+        <v>35</v>
+      </c>
+      <c r="U12" t="s">
+        <v>87</v>
+      </c>
+      <c r="V12" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>